<commit_message>
example plots for Nine-stream-Linnhoff-and-Ahmad
</commit_message>
<xml_diff>
--- a/examples/results/Four-stream-Yee-and-Grossmann-1990-1/Run Metrics.xlsx
+++ b/examples/results/Four-stream-Yee-and-Grossmann-1990-1/Run Metrics.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -519,6 +519,43 @@
         <v>72</v>
       </c>
       <c r="K2" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>25/08/2025 15:41:31</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>154853.8518716671</v>
+      </c>
+      <c r="C3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1210</v>
+      </c>
+      <c r="E3" t="n">
+        <v>112.2966565000825</v>
+      </c>
+      <c r="F3" t="n">
+        <v>154853.8605194094</v>
+      </c>
+      <c r="G3" t="n">
+        <v>159038.7198662622</v>
+      </c>
+      <c r="H3" t="n">
+        <v>163556.1246313013</v>
+      </c>
+      <c r="I3" t="n">
+        <v>34</v>
+      </c>
+      <c r="J3" t="n">
+        <v>72</v>
+      </c>
+      <c r="K3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Restore OpenHENS solver parity
</commit_message>
<xml_diff>
--- a/examples/results/Four-stream-Yee-and-Grossmann-1990-1/Run Metrics.xlsx
+++ b/examples/results/Four-stream-Yee-and-Grossmann-1990-1/Run Metrics.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,61 +413,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Best Solution</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Total Cases Attempted</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Total Cases Solved</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Total Run Time (s)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Quartile 1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Quartile 2</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Quartile 3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Within 2%</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Within 5%</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Within 10%</t>
         </is>
@@ -488,11 +476,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>20/08/2025 17:04:05</t>
+          <t>15/06/2026 15:21:00</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>154853.8518716671</v>
+        <v>154853.8518602861</v>
       </c>
       <c r="C2" t="n">
         <v>1210</v>
@@ -501,61 +489,24 @@
         <v>1210</v>
       </c>
       <c r="E2" t="n">
-        <v>111.9852776000043</v>
+        <v>260.3360324581154</v>
       </c>
       <c r="F2" t="n">
-        <v>154853.8605194094</v>
+        <v>154853.8601589499</v>
       </c>
       <c r="G2" t="n">
-        <v>159038.7198662622</v>
+        <v>159038.7198662623</v>
       </c>
       <c r="H2" t="n">
-        <v>163556.1246313013</v>
+        <v>163556.1251849868</v>
       </c>
       <c r="I2" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="J2" t="n">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="K2" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>25/08/2025 15:41:31</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>154853.8518716671</v>
-      </c>
-      <c r="C3" t="n">
-        <v>1210</v>
-      </c>
-      <c r="D3" t="n">
-        <v>1210</v>
-      </c>
-      <c r="E3" t="n">
-        <v>112.2966565000825</v>
-      </c>
-      <c r="F3" t="n">
-        <v>154853.8605194094</v>
-      </c>
-      <c r="G3" t="n">
-        <v>159038.7198662622</v>
-      </c>
-      <c r="H3" t="n">
-        <v>163556.1246313013</v>
-      </c>
-      <c r="I3" t="n">
-        <v>34</v>
-      </c>
-      <c r="J3" t="n">
-        <v>72</v>
-      </c>
-      <c r="K3" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>